<commit_message>
@faizi968 TOP BOM Updated.
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM (20 Boards).xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SM COM\Desktop\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15480" windowHeight="7872"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="490">
   <si>
     <t>Component list</t>
   </si>
@@ -1485,6 +1485,57 @@
   <si>
     <t>C98220</t>
   </si>
+  <si>
+    <t>Winsource</t>
+  </si>
+  <si>
+    <t>TLV75733PDBVR</t>
+  </si>
+  <si>
+    <t>C485517</t>
+  </si>
+  <si>
+    <t>Design change required. May cause change in some other misc components</t>
+  </si>
+  <si>
+    <t>BD9876AEFJ-E2</t>
+  </si>
+  <si>
+    <t>C79958</t>
+  </si>
+  <si>
+    <t>C100023</t>
+  </si>
+  <si>
+    <t>C516354</t>
+  </si>
+  <si>
+    <t>Need confirmation from client regarding price</t>
+  </si>
+  <si>
+    <t>ISO7221ADR</t>
+  </si>
+  <si>
+    <t>C28037</t>
+  </si>
+  <si>
+    <t>Design change required. May cause change in some other misc components. Quantity also changed from 1/board to 2/board</t>
+  </si>
+  <si>
+    <t>ISO6761FDWR</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>C7042</t>
+  </si>
+  <si>
+    <t>SUM</t>
+  </si>
+  <si>
+    <t>PER BOARD COST</t>
+  </si>
 </sst>
 </file>
 
@@ -1493,7 +1544,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1653,8 +1704,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1694,6 +1753,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1950,7 +2015,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -2165,6 +2230,33 @@
     <xf numFmtId="0" fontId="19" fillId="6" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2174,33 +2266,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2544,26 +2657,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R93"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="30.109375" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="22.109375" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="16.6640625" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="22.140625" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2574,16 +2687,16 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="79"/>
-      <c r="R1" s="79"/>
-    </row>
-    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+    </row>
+    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -2607,7 +2720,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="43"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -2629,9 +2742,9 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="80"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R3" s="89"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -2653,9 +2766,9 @@
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="Q4" s="62"/>
-      <c r="R4" s="81"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R4" s="90"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -2675,9 +2788,9 @@
       <c r="O5" s="62"/>
       <c r="P5" s="62"/>
       <c r="Q5" s="62"/>
-      <c r="R5" s="81"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R5" s="90"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -2695,9 +2808,9 @@
       <c r="O6" s="62"/>
       <c r="P6" s="62"/>
       <c r="Q6" s="62"/>
-      <c r="R6" s="81"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R6" s="90"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -2715,9 +2828,9 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="81"/>
-    </row>
-    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R7" s="90"/>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -2735,9 +2848,9 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="81"/>
-    </row>
-    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R8" s="90"/>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -2791,7 +2904,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -2846,7 +2959,7 @@
       </c>
       <c r="R10" s="41"/>
     </row>
-    <row r="11" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B90" si="0">ROW(B11) - ROW($B$9)</f>
@@ -2901,7 +3014,7 @@
       </c>
       <c r="R11" s="42"/>
     </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -2956,7 +3069,7 @@
       </c>
       <c r="R12" s="41"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
@@ -3011,7 +3124,7 @@
       </c>
       <c r="R13" s="42"/>
     </row>
-    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -3066,7 +3179,7 @@
       </c>
       <c r="R14" s="41"/>
     </row>
-    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
@@ -3121,7 +3234,7 @@
       </c>
       <c r="R15" s="42"/>
     </row>
-    <row r="16" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -3176,7 +3289,7 @@
       </c>
       <c r="R16" s="41"/>
     </row>
-    <row r="17" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f t="shared" si="0"/>
@@ -3231,7 +3344,7 @@
       </c>
       <c r="R17" s="42"/>
     </row>
-    <row r="18" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -3286,7 +3399,7 @@
       </c>
       <c r="R18" s="41"/>
     </row>
-    <row r="19" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f t="shared" si="0"/>
@@ -3341,7 +3454,7 @@
       </c>
       <c r="R19" s="42"/>
     </row>
-    <row r="20" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -3396,7 +3509,7 @@
       </c>
       <c r="R20" s="41"/>
     </row>
-    <row r="21" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f t="shared" si="0"/>
@@ -3451,7 +3564,7 @@
       </c>
       <c r="R21" s="42"/>
     </row>
-    <row r="22" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -3506,7 +3619,7 @@
       </c>
       <c r="R22" s="41"/>
     </row>
-    <row r="23" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f>ROW(B23) - ROW($B$9)</f>
@@ -3561,7 +3674,7 @@
       </c>
       <c r="R23" s="41"/>
     </row>
-    <row r="24" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f t="shared" si="0"/>
@@ -3616,7 +3729,7 @@
       </c>
       <c r="R24" s="42"/>
     </row>
-    <row r="25" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f>ROW(B25) - ROW($B$9)</f>
@@ -3671,7 +3784,7 @@
       </c>
       <c r="R25" s="41"/>
     </row>
-    <row r="26" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f t="shared" si="0"/>
@@ -3726,7 +3839,7 @@
       </c>
       <c r="R26" s="42"/>
     </row>
-    <row r="27" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -3781,7 +3894,7 @@
       </c>
       <c r="R27" s="41"/>
     </row>
-    <row r="28" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f t="shared" si="0"/>
@@ -3836,7 +3949,7 @@
       </c>
       <c r="R28" s="42"/>
     </row>
-    <row r="29" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -3891,7 +4004,7 @@
       </c>
       <c r="R29" s="41"/>
     </row>
-    <row r="30" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f t="shared" si="0"/>
@@ -3946,7 +4059,7 @@
       </c>
       <c r="R30" s="42"/>
     </row>
-    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <f>ROW(B31) - ROW($B$9)</f>
@@ -4001,7 +4114,7 @@
       </c>
       <c r="R31" s="41"/>
     </row>
-    <row r="32" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f t="shared" si="0"/>
@@ -4056,7 +4169,7 @@
       </c>
       <c r="R32" s="42"/>
     </row>
-    <row r="33" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f>ROW(B33) - ROW($B$9)</f>
@@ -4111,7 +4224,7 @@
       </c>
       <c r="R33" s="41"/>
     </row>
-    <row r="34" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f t="shared" si="0"/>
@@ -4166,7 +4279,7 @@
       </c>
       <c r="R34" s="42"/>
     </row>
-    <row r="35" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f>ROW(B35) - ROW($B$9)</f>
@@ -4221,7 +4334,7 @@
       </c>
       <c r="R35" s="41"/>
     </row>
-    <row r="36" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f t="shared" si="0"/>
@@ -4276,7 +4389,7 @@
       </c>
       <c r="R36" s="42"/>
     </row>
-    <row r="37" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f>ROW(B37) - ROW($B$9)</f>
@@ -4331,7 +4444,7 @@
       </c>
       <c r="R37" s="41"/>
     </row>
-    <row r="38" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f t="shared" si="0"/>
@@ -4386,7 +4499,7 @@
       </c>
       <c r="R38" s="42"/>
     </row>
-    <row r="39" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="67">
         <f>ROW(B39) - ROW($B$9)</f>
@@ -4443,7 +4556,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f t="shared" si="0"/>
@@ -4498,7 +4611,7 @@
       </c>
       <c r="R40" s="42"/>
     </row>
-    <row r="41" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f>ROW(B41) - ROW($B$9)</f>
@@ -4553,7 +4666,7 @@
       </c>
       <c r="R41" s="41"/>
     </row>
-    <row r="42" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="67">
         <f t="shared" si="0"/>
@@ -4610,7 +4723,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="67">
         <f>ROW(B43) - ROW($B$9)</f>
@@ -4667,7 +4780,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="53">
         <f t="shared" si="0"/>
@@ -4722,7 +4835,7 @@
       </c>
       <c r="R44" s="42"/>
     </row>
-    <row r="45" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="53">
         <f>ROW(B45) - ROW($B$9)</f>
@@ -4777,7 +4890,7 @@
       </c>
       <c r="R45" s="41"/>
     </row>
-    <row r="46" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="53">
         <f t="shared" si="0"/>
@@ -4832,7 +4945,7 @@
       </c>
       <c r="R46" s="42"/>
     </row>
-    <row r="47" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="53">
         <f>ROW(B47) - ROW($B$9)</f>
@@ -4887,7 +5000,7 @@
       </c>
       <c r="R47" s="41"/>
     </row>
-    <row r="48" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="53">
         <f t="shared" si="0"/>
@@ -4942,7 +5055,7 @@
       </c>
       <c r="R48" s="42"/>
     </row>
-    <row r="49" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="53">
         <f>ROW(B49) - ROW($B$9)</f>
@@ -4997,7 +5110,7 @@
       </c>
       <c r="R49" s="41"/>
     </row>
-    <row r="50" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="53">
         <f t="shared" si="0"/>
@@ -5054,57 +5167,57 @@
         <v>441</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="82">
+      <c r="B51" s="79">
         <f>ROW(B51) - ROW($B$9)</f>
         <v>42</v>
       </c>
-      <c r="C51" s="83" t="s">
+      <c r="C51" s="80" t="s">
         <v>328</v>
       </c>
-      <c r="D51" s="84" t="s">
+      <c r="D51" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="E51" s="85" t="s">
+      <c r="E51" s="82" t="s">
         <v>129</v>
       </c>
-      <c r="F51" s="84" t="s">
+      <c r="F51" s="81" t="s">
         <v>194</v>
       </c>
-      <c r="G51" s="85" t="s">
-        <v>361</v>
-      </c>
-      <c r="H51" s="84" t="s">
-        <v>361</v>
-      </c>
-      <c r="I51" s="84"/>
-      <c r="J51" s="84"/>
-      <c r="K51" s="85" t="s">
-        <v>361</v>
-      </c>
-      <c r="L51" s="84">
+      <c r="G51" s="82" t="s">
+        <v>361</v>
+      </c>
+      <c r="H51" s="81" t="s">
+        <v>361</v>
+      </c>
+      <c r="I51" s="81"/>
+      <c r="J51" s="81"/>
+      <c r="K51" s="82" t="s">
+        <v>361</v>
+      </c>
+      <c r="L51" s="81">
         <v>4</v>
       </c>
-      <c r="M51" s="86">
+      <c r="M51" s="83">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N51" s="86">
-        <f t="shared" ref="N51:N72" si="41">M51+(M51*0.1)</f>
+      <c r="N51" s="83">
+        <f t="shared" ref="N51" si="41">M51+(M51*0.1)</f>
         <v>88</v>
       </c>
-      <c r="O51" s="86"/>
-      <c r="P51" s="86"/>
-      <c r="Q51" s="86">
+      <c r="O51" s="83"/>
+      <c r="P51" s="83"/>
+      <c r="Q51" s="83">
         <f t="shared" ref="Q51" si="42">P51*N51</f>
         <v>0</v>
       </c>
-      <c r="R51" s="90" t="s">
+      <c r="R51" s="87" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="53">
         <f t="shared" si="0"/>
@@ -5161,7 +5274,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="67">
         <f>ROW(B53) - ROW($B$9)</f>
@@ -5194,7 +5307,7 @@
       <c r="K53" s="70" t="s">
         <v>361</v>
       </c>
-      <c r="L53" s="87">
+      <c r="L53" s="84">
         <v>4</v>
       </c>
       <c r="M53" s="71">
@@ -5218,7 +5331,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="53">
         <f t="shared" si="0"/>
@@ -5273,7 +5386,7 @@
       </c>
       <c r="R54" s="42"/>
     </row>
-    <row r="55" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="53">
         <f>ROW(B55) - ROW($B$9)</f>
@@ -5328,7 +5441,7 @@
       </c>
       <c r="R55" s="41"/>
     </row>
-    <row r="56" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="53">
         <f t="shared" si="0"/>
@@ -5383,7 +5496,7 @@
       </c>
       <c r="R56" s="42"/>
     </row>
-    <row r="57" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="53">
         <f>ROW(B57) - ROW($B$9)</f>
@@ -5438,7 +5551,7 @@
       </c>
       <c r="R57" s="41"/>
     </row>
-    <row r="58" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="53">
         <f t="shared" si="0"/>
@@ -5493,7 +5606,7 @@
       </c>
       <c r="R58" s="42"/>
     </row>
-    <row r="59" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="53">
         <f>ROW(B59) - ROW($B$9)</f>
@@ -5548,7 +5661,7 @@
       </c>
       <c r="R59" s="41"/>
     </row>
-    <row r="60" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="53">
         <f t="shared" si="0"/>
@@ -5579,7 +5692,7 @@
       <c r="K60" s="40" t="s">
         <v>335</v>
       </c>
-      <c r="L60" s="89">
+      <c r="L60" s="86">
         <v>9</v>
       </c>
       <c r="M60" s="42">
@@ -5603,7 +5716,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="53">
         <f>ROW(B61) - ROW($B$9)</f>
@@ -5658,7 +5771,7 @@
       </c>
       <c r="R61" s="41"/>
     </row>
-    <row r="62" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="53">
         <f t="shared" si="0"/>
@@ -5713,7 +5826,7 @@
       </c>
       <c r="R62" s="42"/>
     </row>
-    <row r="63" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="53">
         <f>ROW(B63) - ROW($B$9)</f>
@@ -5768,7 +5881,7 @@
       </c>
       <c r="R63" s="41"/>
     </row>
-    <row r="64" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="53">
         <f t="shared" si="0"/>
@@ -5823,7 +5936,7 @@
       </c>
       <c r="R64" s="42"/>
     </row>
-    <row r="65" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="53">
         <f>ROW(B65) - ROW($B$9)</f>
@@ -5878,7 +5991,7 @@
       </c>
       <c r="R65" s="41"/>
     </row>
-    <row r="66" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="53">
         <f t="shared" si="0"/>
@@ -5933,7 +6046,7 @@
       </c>
       <c r="R66" s="42"/>
     </row>
-    <row r="67" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="53">
         <f>ROW(B67) - ROW($B$9)</f>
@@ -5988,7 +6101,7 @@
       </c>
       <c r="R67" s="41"/>
     </row>
-    <row r="68" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="53">
         <f t="shared" si="0"/>
@@ -6043,7 +6156,7 @@
       </c>
       <c r="R68" s="42"/>
     </row>
-    <row r="69" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="53">
         <f>ROW(B69) - ROW($B$9)</f>
@@ -6076,7 +6189,7 @@
       <c r="K69" s="38" t="s">
         <v>344</v>
       </c>
-      <c r="L69" s="88">
+      <c r="L69" s="85">
         <v>2</v>
       </c>
       <c r="M69" s="41">
@@ -6100,7 +6213,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="53">
         <f>ROW(B70) - ROW($B$9)</f>
@@ -6155,7 +6268,7 @@
       </c>
       <c r="R70" s="41"/>
     </row>
-    <row r="71" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="53">
         <f>ROW(B71) - ROW($B$9)</f>
@@ -6210,7 +6323,7 @@
       </c>
       <c r="R71" s="41"/>
     </row>
-    <row r="72" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="53">
         <f t="shared" si="0"/>
@@ -6265,7 +6378,7 @@
       </c>
       <c r="R72" s="42"/>
     </row>
-    <row r="73" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="53">
         <f>ROW(B73) - ROW($B$9)</f>
@@ -6320,7 +6433,7 @@
       </c>
       <c r="R73" s="41"/>
     </row>
-    <row r="74" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="53">
         <f t="shared" si="0"/>
@@ -6375,7 +6488,7 @@
       </c>
       <c r="R74" s="42"/>
     </row>
-    <row r="75" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="53">
         <f>ROW(B75) - ROW($B$9)</f>
@@ -6430,7 +6543,7 @@
       </c>
       <c r="R75" s="41"/>
     </row>
-    <row r="76" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="53">
         <f t="shared" si="0"/>
@@ -6485,7 +6598,7 @@
       </c>
       <c r="R76" s="42"/>
     </row>
-    <row r="77" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="53">
         <f>ROW(B77) - ROW($B$9)</f>
@@ -6540,7 +6653,7 @@
       </c>
       <c r="R77" s="41"/>
     </row>
-    <row r="78" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="53">
         <f t="shared" si="0"/>
@@ -6595,61 +6708,61 @@
       </c>
       <c r="R78" s="42"/>
     </row>
-    <row r="79" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
-      <c r="B79" s="82">
+      <c r="B79" s="79">
         <f>ROW(B79) - ROW($B$9)</f>
         <v>70</v>
       </c>
-      <c r="C79" s="83" t="s">
+      <c r="C79" s="80" t="s">
         <v>201</v>
       </c>
-      <c r="D79" s="84" t="s">
+      <c r="D79" s="81" t="s">
         <v>74</v>
       </c>
-      <c r="E79" s="85" t="s">
+      <c r="E79" s="82" t="s">
         <v>157</v>
       </c>
-      <c r="F79" s="84" t="s">
+      <c r="F79" s="81" t="s">
         <v>201</v>
       </c>
-      <c r="G79" s="85" t="s">
-        <v>361</v>
-      </c>
-      <c r="H79" s="84" t="s">
-        <v>361</v>
-      </c>
-      <c r="I79" s="84" t="s">
-        <v>361</v>
-      </c>
-      <c r="J79" s="84" t="s">
-        <v>361</v>
-      </c>
-      <c r="K79" s="85" t="s">
-        <v>361</v>
-      </c>
-      <c r="L79" s="84">
+      <c r="G79" s="82" t="s">
+        <v>361</v>
+      </c>
+      <c r="H79" s="81" t="s">
+        <v>361</v>
+      </c>
+      <c r="I79" s="81" t="s">
+        <v>361</v>
+      </c>
+      <c r="J79" s="81" t="s">
+        <v>361</v>
+      </c>
+      <c r="K79" s="82" t="s">
+        <v>361</v>
+      </c>
+      <c r="L79" s="81">
         <v>11</v>
       </c>
-      <c r="M79" s="86">
+      <c r="M79" s="83">
         <f t="shared" si="64"/>
         <v>220</v>
       </c>
-      <c r="N79" s="86">
-        <f t="shared" ref="N73:N91" si="71">M79+(M79*0.1)</f>
+      <c r="N79" s="83">
+        <f t="shared" ref="N79:N91" si="71">M79+(M79*0.1)</f>
         <v>242</v>
       </c>
-      <c r="O79" s="86"/>
-      <c r="P79" s="86"/>
-      <c r="Q79" s="86">
+      <c r="O79" s="83"/>
+      <c r="P79" s="83"/>
+      <c r="Q79" s="83">
         <f t="shared" ref="Q79" si="72">P79*N79</f>
         <v>0</v>
       </c>
-      <c r="R79" s="90" t="s">
+      <c r="R79" s="87" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="53">
         <f t="shared" si="0"/>
@@ -6699,7 +6812,7 @@
       </c>
       <c r="R80" s="42"/>
     </row>
-    <row r="81" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="53">
         <f>ROW(B81) - ROW($B$9)</f>
@@ -6723,8 +6836,12 @@
       <c r="H81" s="37" t="s">
         <v>296</v>
       </c>
-      <c r="I81" s="37"/>
-      <c r="J81" s="37"/>
+      <c r="I81" s="37" t="s">
+        <v>361</v>
+      </c>
+      <c r="J81" s="37" t="s">
+        <v>361</v>
+      </c>
       <c r="K81" s="38" t="s">
         <v>361</v>
       </c>
@@ -6736,18 +6853,21 @@
         <v>20</v>
       </c>
       <c r="N81" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O81" s="41"/>
-      <c r="P81" s="41"/>
+        <v>21</v>
+      </c>
+      <c r="O81" s="64" t="s">
+        <v>435</v>
+      </c>
+      <c r="P81" s="41">
+        <v>3.81</v>
+      </c>
       <c r="Q81" s="41">
         <f t="shared" ref="Q81" si="74">P81*N81</f>
-        <v>0</v>
+        <v>80.010000000000005</v>
       </c>
       <c r="R81" s="41"/>
     </row>
-    <row r="82" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="53">
         <f t="shared" si="0"/>
@@ -6790,111 +6910,133 @@
       <c r="N82" s="42">
         <v>21</v>
       </c>
-      <c r="O82" s="42"/>
-      <c r="P82" s="42"/>
+      <c r="O82" s="65" t="s">
+        <v>473</v>
+      </c>
+      <c r="P82" s="42">
+        <v>2.48</v>
+      </c>
       <c r="Q82" s="42">
         <f t="shared" ref="Q82" si="75">N82*P82</f>
-        <v>0</v>
+        <v>52.08</v>
       </c>
       <c r="R82" s="42"/>
     </row>
-    <row r="83" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
-      <c r="B83" s="53">
+      <c r="B83" s="91">
         <f>ROW(B83) - ROW($B$9)</f>
         <v>74</v>
       </c>
-      <c r="C83" s="61" t="s">
+      <c r="C83" s="92" t="s">
         <v>376</v>
       </c>
-      <c r="D83" s="37" t="s">
+      <c r="D83" s="93" t="s">
         <v>78</v>
       </c>
-      <c r="E83" s="38" t="s">
+      <c r="E83" s="94" t="s">
         <v>161</v>
       </c>
-      <c r="F83" s="37" t="s">
+      <c r="F83" s="93" t="s">
         <v>204</v>
       </c>
-      <c r="G83" s="38" t="s">
+      <c r="G83" s="94" t="s">
         <v>261</v>
       </c>
-      <c r="H83" s="37" t="s">
+      <c r="H83" s="93" t="s">
         <v>298</v>
       </c>
-      <c r="I83" s="37"/>
-      <c r="J83" s="37"/>
-      <c r="K83" s="38" t="s">
-        <v>361</v>
-      </c>
-      <c r="L83" s="37">
+      <c r="I83" s="93" t="s">
+        <v>474</v>
+      </c>
+      <c r="J83" s="93" t="s">
+        <v>475</v>
+      </c>
+      <c r="K83" s="94" t="s">
+        <v>361</v>
+      </c>
+      <c r="L83" s="93">
         <v>1</v>
       </c>
-      <c r="M83" s="41">
+      <c r="M83" s="95">
         <f t="shared" si="64"/>
         <v>20</v>
       </c>
-      <c r="N83" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O83" s="41"/>
-      <c r="P83" s="41"/>
-      <c r="Q83" s="41">
+      <c r="N83" s="95">
+        <v>21</v>
+      </c>
+      <c r="O83" s="96" t="s">
+        <v>391</v>
+      </c>
+      <c r="P83" s="95">
+        <v>1.3939999999999999</v>
+      </c>
+      <c r="Q83" s="95">
         <f t="shared" ref="Q83" si="76">P83*N83</f>
-        <v>0</v>
-      </c>
-      <c r="R83" s="41"/>
-    </row>
-    <row r="84" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+        <v>29.273999999999997</v>
+      </c>
+      <c r="R83" s="97" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="84" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
-      <c r="B84" s="53">
+      <c r="B84" s="91">
         <f t="shared" si="0"/>
         <v>75</v>
       </c>
-      <c r="C84" s="60" t="s">
+      <c r="C84" s="98" t="s">
         <v>376</v>
       </c>
-      <c r="D84" s="39" t="s">
+      <c r="D84" s="99" t="s">
         <v>79</v>
       </c>
-      <c r="E84" s="40" t="s">
+      <c r="E84" s="100" t="s">
         <v>162</v>
       </c>
-      <c r="F84" s="39" t="s">
+      <c r="F84" s="99" t="s">
         <v>205</v>
       </c>
-      <c r="G84" s="40" t="s">
+      <c r="G84" s="100" t="s">
         <v>262</v>
       </c>
-      <c r="H84" s="39" t="s">
+      <c r="H84" s="99" t="s">
         <v>297</v>
       </c>
-      <c r="I84" s="39"/>
-      <c r="J84" s="39"/>
-      <c r="K84" s="40" t="s">
-        <v>361</v>
-      </c>
-      <c r="L84" s="39">
+      <c r="I84" s="99" t="s">
+        <v>477</v>
+      </c>
+      <c r="J84" s="99" t="s">
+        <v>478</v>
+      </c>
+      <c r="K84" s="100" t="s">
+        <v>361</v>
+      </c>
+      <c r="L84" s="99">
         <v>1</v>
       </c>
-      <c r="M84" s="42">
+      <c r="M84" s="101">
         <f t="shared" si="64"/>
         <v>20</v>
       </c>
-      <c r="N84" s="42">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O84" s="42"/>
-      <c r="P84" s="42"/>
-      <c r="Q84" s="42">
+      <c r="N84" s="101">
+        <v>21</v>
+      </c>
+      <c r="O84" s="102" t="s">
+        <v>391</v>
+      </c>
+      <c r="P84" s="101">
+        <v>0.69430000000000003</v>
+      </c>
+      <c r="Q84" s="101">
         <f t="shared" ref="Q84" si="77">N84*P84</f>
-        <v>0</v>
-      </c>
-      <c r="R84" s="42"/>
-    </row>
-    <row r="85" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>14.580300000000001</v>
+      </c>
+      <c r="R84" s="97" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="53">
         <f>ROW(B85) - ROW($B$9)</f>
@@ -6918,8 +7060,12 @@
       <c r="H85" s="37" t="s">
         <v>297</v>
       </c>
-      <c r="I85" s="37"/>
-      <c r="J85" s="37"/>
+      <c r="I85" s="37" t="s">
+        <v>361</v>
+      </c>
+      <c r="J85" s="37" t="s">
+        <v>361</v>
+      </c>
       <c r="K85" s="38" t="s">
         <v>361</v>
       </c>
@@ -6931,18 +7077,21 @@
         <v>20</v>
       </c>
       <c r="N85" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O85" s="41"/>
-      <c r="P85" s="41"/>
+        <v>21</v>
+      </c>
+      <c r="O85" s="64" t="s">
+        <v>473</v>
+      </c>
+      <c r="P85" s="41">
+        <v>3.637</v>
+      </c>
       <c r="Q85" s="41">
         <f t="shared" ref="Q85" si="78">P85*N85</f>
-        <v>0</v>
+        <v>76.376999999999995</v>
       </c>
       <c r="R85" s="41"/>
     </row>
-    <row r="86" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
       <c r="B86" s="53">
         <f t="shared" si="0"/>
@@ -6966,8 +7115,12 @@
       <c r="H86" s="39" t="s">
         <v>297</v>
       </c>
-      <c r="I86" s="39"/>
-      <c r="J86" s="39"/>
+      <c r="I86" s="39" t="s">
+        <v>361</v>
+      </c>
+      <c r="J86" s="39" t="s">
+        <v>479</v>
+      </c>
       <c r="K86" s="40" t="s">
         <v>361</v>
       </c>
@@ -6979,66 +7132,78 @@
         <v>20</v>
       </c>
       <c r="N86" s="42">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O86" s="42"/>
-      <c r="P86" s="42"/>
+        <v>21</v>
+      </c>
+      <c r="O86" s="65" t="s">
+        <v>391</v>
+      </c>
+      <c r="P86" s="42">
+        <v>0.43280000000000002</v>
+      </c>
       <c r="Q86" s="42">
         <f t="shared" ref="Q86" si="79">N86*P86</f>
-        <v>0</v>
+        <v>9.0888000000000009</v>
       </c>
       <c r="R86" s="42"/>
     </row>
-    <row r="87" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
-      <c r="B87" s="53">
+      <c r="B87" s="91">
         <f>ROW(B87) - ROW($B$9)</f>
         <v>78</v>
       </c>
-      <c r="C87" s="61" t="s">
+      <c r="C87" s="92" t="s">
         <v>376</v>
       </c>
-      <c r="D87" s="37" t="s">
+      <c r="D87" s="93" t="s">
         <v>82</v>
       </c>
-      <c r="E87" s="38" t="s">
+      <c r="E87" s="94" t="s">
         <v>165</v>
       </c>
-      <c r="F87" s="37" t="s">
+      <c r="F87" s="93" t="s">
         <v>208</v>
       </c>
-      <c r="G87" s="38" t="s">
+      <c r="G87" s="94" t="s">
         <v>264</v>
       </c>
-      <c r="H87" s="37" t="s">
+      <c r="H87" s="93" t="s">
         <v>299</v>
       </c>
-      <c r="I87" s="37"/>
-      <c r="J87" s="37"/>
-      <c r="K87" s="38" t="s">
-        <v>361</v>
-      </c>
-      <c r="L87" s="37">
+      <c r="I87" s="93" t="s">
+        <v>361</v>
+      </c>
+      <c r="J87" s="93" t="s">
+        <v>480</v>
+      </c>
+      <c r="K87" s="94" t="s">
+        <v>361</v>
+      </c>
+      <c r="L87" s="93">
         <v>1</v>
       </c>
-      <c r="M87" s="41">
+      <c r="M87" s="95">
         <f t="shared" si="64"/>
         <v>20</v>
       </c>
-      <c r="N87" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O87" s="41"/>
-      <c r="P87" s="41"/>
-      <c r="Q87" s="41">
+      <c r="N87" s="95">
+        <v>21</v>
+      </c>
+      <c r="O87" s="96" t="s">
+        <v>391</v>
+      </c>
+      <c r="P87" s="95">
+        <v>7.4638</v>
+      </c>
+      <c r="Q87" s="95">
         <f t="shared" ref="Q87" si="80">P87*N87</f>
-        <v>0</v>
-      </c>
-      <c r="R87" s="41"/>
-    </row>
-    <row r="88" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>156.7398</v>
+      </c>
+      <c r="R87" s="95" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="53">
         <f t="shared" si="0"/>
@@ -7062,8 +7227,12 @@
       <c r="H88" s="39" t="s">
         <v>300</v>
       </c>
-      <c r="I88" s="39"/>
-      <c r="J88" s="39"/>
+      <c r="I88" s="39" t="s">
+        <v>361</v>
+      </c>
+      <c r="J88" s="39" t="s">
+        <v>361</v>
+      </c>
       <c r="K88" s="58" t="s">
         <v>362</v>
       </c>
@@ -7075,114 +7244,135 @@
         <v>20</v>
       </c>
       <c r="N88" s="42">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O88" s="42"/>
-      <c r="P88" s="42"/>
+        <v>21</v>
+      </c>
+      <c r="O88" s="65" t="s">
+        <v>473</v>
+      </c>
+      <c r="P88" s="42">
+        <v>2.6459999999999999</v>
+      </c>
       <c r="Q88" s="42">
         <f t="shared" ref="Q88" si="81">N88*P88</f>
-        <v>0</v>
+        <v>55.565999999999995</v>
       </c>
       <c r="R88" s="42"/>
     </row>
-    <row r="89" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="53">
+      <c r="B89" s="91">
         <f>ROW(B89) - ROW($B$9)</f>
         <v>80</v>
       </c>
-      <c r="C89" s="61" t="s">
+      <c r="C89" s="92" t="s">
         <v>376</v>
       </c>
-      <c r="D89" s="37" t="s">
+      <c r="D89" s="93" t="s">
         <v>84</v>
       </c>
-      <c r="E89" s="38" t="s">
+      <c r="E89" s="94" t="s">
         <v>167</v>
       </c>
-      <c r="F89" s="37" t="s">
+      <c r="F89" s="93" t="s">
         <v>358</v>
       </c>
-      <c r="G89" s="38" t="s">
+      <c r="G89" s="94" t="s">
         <v>210</v>
       </c>
-      <c r="H89" s="37" t="s">
+      <c r="H89" s="93" t="s">
         <v>297</v>
       </c>
-      <c r="I89" s="37"/>
-      <c r="J89" s="37"/>
-      <c r="K89" s="38" t="s">
-        <v>361</v>
-      </c>
-      <c r="L89" s="37">
+      <c r="I89" s="93" t="s">
+        <v>482</v>
+      </c>
+      <c r="J89" s="93" t="s">
+        <v>483</v>
+      </c>
+      <c r="K89" s="94" t="s">
+        <v>361</v>
+      </c>
+      <c r="L89" s="103">
+        <v>2</v>
+      </c>
+      <c r="M89" s="95">
+        <f t="shared" si="64"/>
+        <v>40</v>
+      </c>
+      <c r="N89" s="95">
+        <v>42</v>
+      </c>
+      <c r="O89" s="96" t="s">
+        <v>391</v>
+      </c>
+      <c r="P89" s="95">
+        <v>2.2974000000000001</v>
+      </c>
+      <c r="Q89" s="95">
+        <f t="shared" ref="Q89" si="82">P89*N89</f>
+        <v>96.490800000000007</v>
+      </c>
+      <c r="R89" s="97" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="1"/>
+      <c r="B90" s="91">
+        <f t="shared" si="0"/>
+        <v>81</v>
+      </c>
+      <c r="C90" s="98" t="s">
+        <v>376</v>
+      </c>
+      <c r="D90" s="99" t="s">
+        <v>85</v>
+      </c>
+      <c r="E90" s="100" t="s">
+        <v>168</v>
+      </c>
+      <c r="F90" s="99" t="s">
+        <v>359</v>
+      </c>
+      <c r="G90" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="H90" s="99" t="s">
+        <v>300</v>
+      </c>
+      <c r="I90" s="99" t="s">
+        <v>485</v>
+      </c>
+      <c r="J90" s="99" t="s">
+        <v>361</v>
+      </c>
+      <c r="K90" s="100" t="s">
+        <v>361</v>
+      </c>
+      <c r="L90" s="99">
         <v>1</v>
       </c>
-      <c r="M89" s="41">
+      <c r="M90" s="101">
         <f t="shared" si="64"/>
         <v>20</v>
       </c>
-      <c r="N89" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O89" s="41"/>
-      <c r="P89" s="41"/>
-      <c r="Q89" s="41">
-        <f t="shared" ref="Q89" si="82">P89*N89</f>
-        <v>0</v>
-      </c>
-      <c r="R89" s="41"/>
-    </row>
-    <row r="90" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A90" s="1"/>
-      <c r="B90" s="53">
-        <f t="shared" si="0"/>
-        <v>81</v>
-      </c>
-      <c r="C90" s="60" t="s">
-        <v>376</v>
-      </c>
-      <c r="D90" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="E90" s="40" t="s">
-        <v>168</v>
-      </c>
-      <c r="F90" s="39" t="s">
-        <v>359</v>
-      </c>
-      <c r="G90" s="40" t="s">
-        <v>211</v>
-      </c>
-      <c r="H90" s="39" t="s">
-        <v>300</v>
-      </c>
-      <c r="I90" s="39"/>
-      <c r="J90" s="39"/>
-      <c r="K90" s="40" t="s">
-        <v>361</v>
-      </c>
-      <c r="L90" s="39">
-        <v>1</v>
-      </c>
-      <c r="M90" s="42">
-        <f t="shared" si="64"/>
-        <v>20</v>
-      </c>
-      <c r="N90" s="42">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O90" s="42"/>
-      <c r="P90" s="42"/>
-      <c r="Q90" s="42">
+      <c r="N90" s="101">
+        <v>21</v>
+      </c>
+      <c r="O90" s="102" t="s">
+        <v>486</v>
+      </c>
+      <c r="P90" s="101">
+        <v>3.532</v>
+      </c>
+      <c r="Q90" s="101">
         <f t="shared" ref="Q90" si="83">N90*P90</f>
-        <v>0</v>
-      </c>
-      <c r="R90" s="42"/>
-    </row>
-    <row r="91" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>74.171999999999997</v>
+      </c>
+      <c r="R90" s="97" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
       <c r="B91" s="53">
         <f>ROW(B91) - ROW($B$9)</f>
@@ -7206,8 +7396,12 @@
       <c r="H91" s="37" t="s">
         <v>297</v>
       </c>
-      <c r="I91" s="63"/>
-      <c r="J91" s="63"/>
+      <c r="I91" s="63" t="s">
+        <v>361</v>
+      </c>
+      <c r="J91" s="63" t="s">
+        <v>487</v>
+      </c>
       <c r="K91" s="38" t="s">
         <v>361</v>
       </c>
@@ -7219,18 +7413,21 @@
         <v>20</v>
       </c>
       <c r="N91" s="41">
-        <f t="shared" si="71"/>
-        <v>22</v>
-      </c>
-      <c r="O91" s="41"/>
-      <c r="P91" s="41"/>
+        <v>21</v>
+      </c>
+      <c r="O91" s="64" t="s">
+        <v>391</v>
+      </c>
+      <c r="P91" s="41">
+        <v>0.39140000000000003</v>
+      </c>
       <c r="Q91" s="41">
         <f t="shared" ref="Q91" si="84">P91*N91</f>
-        <v>0</v>
+        <v>8.2194000000000003</v>
       </c>
       <c r="R91" s="41"/>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="32"/>
       <c r="C92" s="51"/>
@@ -7247,12 +7444,20 @@
       <c r="L92" s="36"/>
       <c r="M92" s="36"/>
       <c r="N92" s="36"/>
-      <c r="O92" s="36"/>
-      <c r="P92" s="36"/>
-      <c r="Q92" s="36"/>
+      <c r="O92" s="106" t="s">
+        <v>488</v>
+      </c>
+      <c r="P92" s="104">
+        <f>SUM(P10:P91)</f>
+        <v>37.098149999999997</v>
+      </c>
+      <c r="Q92" s="104">
+        <f>SUM(Q10:Q91)</f>
+        <v>976.02435000000014</v>
+      </c>
       <c r="R92" s="44"/>
     </row>
-    <row r="93" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
       <c r="B93" s="24"/>
       <c r="C93" s="52"/>
@@ -7269,9 +7474,14 @@
       <c r="L93" s="9"/>
       <c r="M93" s="9"/>
       <c r="N93" s="9"/>
-      <c r="O93" s="9"/>
-      <c r="P93" s="9"/>
-      <c r="Q93" s="9"/>
+      <c r="O93" s="107" t="s">
+        <v>489</v>
+      </c>
+      <c r="P93" s="105"/>
+      <c r="Q93" s="105">
+        <f>Q92/20</f>
+        <v>48.801217500000007</v>
+      </c>
       <c r="R93" s="45"/>
     </row>
   </sheetData>
@@ -7348,9 +7558,20 @@
     <hyperlink ref="O76" r:id="rId66"/>
     <hyperlink ref="O77" r:id="rId67"/>
     <hyperlink ref="O78" r:id="rId68"/>
+    <hyperlink ref="O81" r:id="rId69"/>
+    <hyperlink ref="O82" r:id="rId70"/>
+    <hyperlink ref="O83" r:id="rId71"/>
+    <hyperlink ref="O84" r:id="rId72"/>
+    <hyperlink ref="O85" r:id="rId73"/>
+    <hyperlink ref="O86" r:id="rId74"/>
+    <hyperlink ref="O87" r:id="rId75"/>
+    <hyperlink ref="O88" r:id="rId76"/>
+    <hyperlink ref="O89" r:id="rId77"/>
+    <hyperlink ref="O90" r:id="rId78"/>
+    <hyperlink ref="O91" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId69"/>
-  <drawing r:id="rId70"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId80"/>
+  <drawing r:id="rId81"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BOM and schematic changes #135
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/eSpark BOM (20 Boards).xlsx
+++ b/Deliverables/SM_Top Board/_BOM/eSpark BOM (20 Boards).xlsx
@@ -1653,22 +1653,6 @@
     <t>Quantity changed from 3/board to 1/board due to removal of two capacitors after changes in circuitry of U3</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">C8, C10, C11, C12, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>C41</t>
-    </r>
-  </si>
-  <si>
     <t>GRM188R6YA106MA73D</t>
   </si>
   <si>
@@ -1698,9 +1682,6 @@
   </si>
   <si>
     <t>C194427</t>
-  </si>
-  <si>
-    <t>Quantity changed from 4/board to 5/board due to addition of 1 x 10uF capacitor from U3</t>
   </si>
   <si>
     <r>
@@ -1942,6 +1923,25 @@
   </si>
   <si>
     <t>Will be provided by Robotshop for prototyping</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">C8, C10, C11, C12, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C41, CF3</t>
+    </r>
+  </si>
+  <si>
+    <t>Quantity changed from 4/board to 6/board due to addition of 2 x 10uF capacitor from U3</t>
   </si>
 </sst>
 </file>
@@ -2471,7 +2471,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -2740,9 +2740,6 @@
     <xf numFmtId="0" fontId="19" fillId="8" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2752,6 +2749,63 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2761,109 +2815,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3239,14 +3257,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="102"/>
-      <c r="L1" s="102"/>
-      <c r="M1" s="102"/>
-      <c r="N1" s="102"/>
-      <c r="O1" s="102"/>
-      <c r="P1" s="102"/>
-      <c r="Q1" s="102"/>
-      <c r="R1" s="102"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
     </row>
     <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -3294,7 +3312,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="103"/>
+      <c r="R3" s="121"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -3318,7 +3336,7 @@
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="Q4" s="62"/>
-      <c r="R4" s="104"/>
+      <c r="R4" s="122"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -3340,7 +3358,7 @@
       <c r="O5" s="62"/>
       <c r="P5" s="62"/>
       <c r="Q5" s="62"/>
-      <c r="R5" s="104"/>
+      <c r="R5" s="122"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -3360,7 +3378,7 @@
       <c r="O6" s="62"/>
       <c r="P6" s="62"/>
       <c r="Q6" s="62"/>
-      <c r="R6" s="104"/>
+      <c r="R6" s="122"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -3380,7 +3398,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="104"/>
+      <c r="R7" s="122"/>
     </row>
     <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
@@ -3400,7 +3418,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="104"/>
+      <c r="R8" s="122"/>
     </row>
     <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
@@ -3568,287 +3586,287 @@
     </row>
     <row r="12" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
-      <c r="B12" s="85">
+      <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="86" t="s">
+      <c r="C12" s="61" t="s">
         <v>341</v>
       </c>
-      <c r="D12" s="87" t="s">
+      <c r="D12" s="37" t="s">
         <v>478</v>
       </c>
-      <c r="E12" s="88" t="s">
+      <c r="E12" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="87" t="s">
+      <c r="F12" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="G12" s="88" t="s">
+      <c r="G12" s="38" t="s">
         <v>199</v>
       </c>
-      <c r="H12" s="87" t="s">
+      <c r="H12" s="37" t="s">
         <v>250</v>
       </c>
-      <c r="I12" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J12" s="87" t="s">
+      <c r="I12" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J12" s="37" t="s">
         <v>370</v>
       </c>
-      <c r="K12" s="88" t="s">
+      <c r="K12" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="L12" s="109">
+      <c r="L12" s="123">
         <v>2</v>
       </c>
-      <c r="M12" s="89">
+      <c r="M12" s="41">
         <f t="shared" ref="M12:M73" si="1">L12*20</f>
         <v>40</v>
       </c>
-      <c r="N12" s="89">
+      <c r="N12" s="41">
         <v>100</v>
       </c>
-      <c r="O12" s="90" t="s">
+      <c r="O12" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P12" s="89">
+      <c r="P12" s="41">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="Q12" s="89">
+      <c r="Q12" s="41">
         <f t="shared" ref="Q12" si="2">P12*N12</f>
         <v>0.13</v>
       </c>
-      <c r="R12" s="106" t="s">
+      <c r="R12" s="124" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
-      <c r="B13" s="85">
+      <c r="B13" s="53">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="92" t="s">
+      <c r="C13" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="D13" s="93" t="s">
+      <c r="D13" s="39" t="s">
         <v>477</v>
       </c>
-      <c r="E13" s="94" t="s">
+      <c r="E13" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="93" t="s">
+      <c r="F13" s="39" t="s">
         <v>159</v>
       </c>
-      <c r="G13" s="94" t="s">
+      <c r="G13" s="40" t="s">
         <v>200</v>
       </c>
-      <c r="H13" s="93" t="s">
+      <c r="H13" s="39" t="s">
         <v>251</v>
       </c>
-      <c r="I13" s="93" t="s">
-        <v>338</v>
-      </c>
-      <c r="J13" s="93" t="s">
+      <c r="I13" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="J13" s="39" t="s">
         <v>371</v>
       </c>
-      <c r="K13" s="94" t="s">
+      <c r="K13" s="40" t="s">
         <v>285</v>
       </c>
-      <c r="L13" s="108">
+      <c r="L13" s="127">
         <v>1</v>
       </c>
-      <c r="M13" s="95">
+      <c r="M13" s="42">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N13" s="107">
+      <c r="N13" s="128">
         <v>40</v>
       </c>
-      <c r="O13" s="96" t="s">
+      <c r="O13" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P13" s="95">
+      <c r="P13" s="42">
         <v>3.5900000000000001E-2</v>
       </c>
-      <c r="Q13" s="95">
+      <c r="Q13" s="42">
         <f t="shared" ref="Q13" si="3">N13*P13</f>
         <v>1.4359999999999999</v>
       </c>
-      <c r="R13" s="106" t="s">
+      <c r="R13" s="129" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="85">
+      <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="86" t="s">
+      <c r="C14" s="61" t="s">
         <v>341</v>
       </c>
-      <c r="D14" s="87" t="s">
+      <c r="D14" s="37" t="s">
         <v>475</v>
       </c>
-      <c r="E14" s="88" t="s">
+      <c r="E14" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="87" t="s">
+      <c r="F14" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="G14" s="88" t="s">
+      <c r="G14" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H14" s="87" t="s">
+      <c r="H14" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="I14" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J14" s="87" t="s">
+      <c r="I14" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J14" s="37" t="s">
         <v>372</v>
       </c>
-      <c r="K14" s="88" t="s">
+      <c r="K14" s="38" t="s">
         <v>286</v>
       </c>
-      <c r="L14" s="87">
+      <c r="L14" s="37">
         <v>8</v>
       </c>
-      <c r="M14" s="89">
+      <c r="M14" s="41">
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="N14" s="89">
+      <c r="N14" s="41">
         <v>200</v>
       </c>
-      <c r="O14" s="90" t="s">
+      <c r="O14" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P14" s="89">
+      <c r="P14" s="41">
         <v>4.0899999999999999E-2</v>
       </c>
-      <c r="Q14" s="89">
+      <c r="Q14" s="41">
         <f>P14*N14</f>
         <v>8.18</v>
       </c>
-      <c r="R14" s="106" t="s">
+      <c r="R14" s="124" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
-      <c r="B15" s="85">
+      <c r="B15" s="53">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="92" t="s">
+      <c r="C15" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="D15" s="93" t="s">
+      <c r="D15" s="39" t="s">
         <v>471</v>
       </c>
-      <c r="E15" s="94" t="s">
+      <c r="E15" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="F15" s="93" t="s">
+      <c r="F15" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="G15" s="94" t="s">
+      <c r="G15" s="40" t="s">
         <v>202</v>
       </c>
-      <c r="H15" s="93" t="s">
+      <c r="H15" s="39" t="s">
         <v>250</v>
       </c>
-      <c r="I15" s="93" t="s">
-        <v>338</v>
-      </c>
-      <c r="J15" s="93" t="s">
+      <c r="I15" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="J15" s="39" t="s">
         <v>373</v>
       </c>
-      <c r="K15" s="94" t="s">
+      <c r="K15" s="40" t="s">
         <v>287</v>
       </c>
-      <c r="L15" s="108">
+      <c r="L15" s="127">
         <v>3</v>
       </c>
-      <c r="M15" s="95">
+      <c r="M15" s="42">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="N15" s="107">
+      <c r="N15" s="128">
         <v>100</v>
       </c>
-      <c r="O15" s="96" t="s">
+      <c r="O15" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P15" s="95">
+      <c r="P15" s="42">
         <v>5.8999999999999999E-3</v>
       </c>
-      <c r="Q15" s="95">
+      <c r="Q15" s="42">
         <f t="shared" ref="Q15" si="4">N15*P15</f>
         <v>0.59</v>
       </c>
-      <c r="R15" s="106" t="s">
+      <c r="R15" s="129" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
-      <c r="B16" s="85">
+      <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="86" t="s">
+      <c r="C16" s="61" t="s">
         <v>341</v>
       </c>
-      <c r="D16" s="87" t="s">
+      <c r="D16" s="37" t="s">
+        <v>511</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>491</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="G16" s="125" t="s">
         <v>490</v>
       </c>
-      <c r="E16" s="88" t="s">
+      <c r="H16" s="126" t="s">
+        <v>252</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J16" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="F16" s="87" t="s">
-        <v>158</v>
-      </c>
-      <c r="G16" s="132" t="s">
-        <v>491</v>
-      </c>
-      <c r="H16" s="97" t="s">
-        <v>252</v>
-      </c>
-      <c r="I16" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J16" s="87" t="s">
-        <v>493</v>
-      </c>
-      <c r="K16" s="88" t="s">
+      <c r="K16" s="38" t="s">
         <v>288</v>
       </c>
-      <c r="L16" s="87">
-        <v>5</v>
-      </c>
-      <c r="M16" s="89">
+      <c r="L16" s="37">
+        <v>6</v>
+      </c>
+      <c r="M16" s="41">
         <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="N16" s="89">
-        <v>110</v>
-      </c>
-      <c r="O16" s="90" t="s">
+        <v>120</v>
+      </c>
+      <c r="N16" s="41">
+        <v>130</v>
+      </c>
+      <c r="O16" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P16" s="89">
+      <c r="P16" s="41">
         <v>3.32E-2</v>
       </c>
-      <c r="Q16" s="89">
+      <c r="Q16" s="41">
         <f t="shared" ref="Q16" si="5">P16*N16</f>
-        <v>3.6520000000000001</v>
-      </c>
-      <c r="R16" s="106" t="s">
-        <v>494</v>
+        <v>4.3159999999999998</v>
+      </c>
+      <c r="R16" s="124" t="s">
+        <v>512</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -4238,58 +4256,58 @@
     </row>
     <row r="24" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
-      <c r="B24" s="85">
+      <c r="B24" s="53">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="92" t="s">
+      <c r="C24" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="D24" s="93" t="s">
+      <c r="D24" s="39" t="s">
         <v>468</v>
       </c>
-      <c r="E24" s="94" t="s">
+      <c r="E24" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="F24" s="93" t="s">
+      <c r="F24" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="G24" s="94" t="s">
+      <c r="G24" s="40" t="s">
         <v>209</v>
       </c>
-      <c r="H24" s="93" t="s">
+      <c r="H24" s="39" t="s">
         <v>249</v>
       </c>
-      <c r="I24" s="93" t="s">
-        <v>338</v>
-      </c>
-      <c r="J24" s="93" t="s">
+      <c r="I24" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="J24" s="39" t="s">
         <v>384</v>
       </c>
-      <c r="K24" s="94" t="s">
+      <c r="K24" s="40" t="s">
         <v>293</v>
       </c>
-      <c r="L24" s="108">
+      <c r="L24" s="127">
         <v>1</v>
       </c>
-      <c r="M24" s="95">
+      <c r="M24" s="42">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N24" s="107">
+      <c r="N24" s="128">
         <v>40</v>
       </c>
-      <c r="O24" s="96" t="s">
+      <c r="O24" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P24" s="95">
+      <c r="P24" s="42">
         <v>1.9199999999999998E-2</v>
       </c>
-      <c r="Q24" s="95">
+      <c r="Q24" s="42">
         <f t="shared" ref="Q24" si="13">N24*P24</f>
         <v>0.7679999999999999</v>
       </c>
-      <c r="R24" s="106" t="s">
+      <c r="R24" s="129" t="s">
         <v>469</v>
       </c>
     </row>
@@ -4405,229 +4423,229 @@
     </row>
     <row r="27" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
-      <c r="B27" s="113">
+      <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="133" t="s">
+      <c r="C27" s="130" t="s">
         <v>341</v>
       </c>
-      <c r="D27" s="134" t="s">
+      <c r="D27" s="131" t="s">
         <v>18</v>
       </c>
-      <c r="E27" s="135" t="s">
+      <c r="E27" s="132" t="s">
         <v>94</v>
       </c>
-      <c r="F27" s="134" t="s">
+      <c r="F27" s="131" t="s">
         <v>162</v>
       </c>
-      <c r="G27" s="135" t="s">
+      <c r="G27" s="132" t="s">
         <v>211</v>
       </c>
-      <c r="H27" s="134" t="s">
+      <c r="H27" s="131" t="s">
         <v>251</v>
       </c>
-      <c r="I27" s="134" t="s">
-        <v>338</v>
-      </c>
-      <c r="J27" s="134" t="s">
+      <c r="I27" s="131" t="s">
+        <v>338</v>
+      </c>
+      <c r="J27" s="131" t="s">
         <v>388</v>
       </c>
-      <c r="K27" s="135" t="s">
+      <c r="K27" s="132" t="s">
         <v>296</v>
       </c>
-      <c r="L27" s="134">
+      <c r="L27" s="131">
         <v>1</v>
       </c>
-      <c r="M27" s="136">
+      <c r="M27" s="133">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N27" s="136">
+      <c r="N27" s="133">
         <v>0</v>
       </c>
-      <c r="O27" s="137" t="s">
+      <c r="O27" s="134" t="s">
         <v>368</v>
       </c>
-      <c r="P27" s="136">
+      <c r="P27" s="133">
         <v>0.1653</v>
       </c>
-      <c r="Q27" s="136">
+      <c r="Q27" s="133">
         <f t="shared" ref="Q27" si="16">P27*N27</f>
         <v>0</v>
       </c>
-      <c r="R27" s="136" t="s">
+      <c r="R27" s="133" t="s">
         <v>481</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
-      <c r="B28" s="85">
+      <c r="B28" s="53">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="92" t="s">
+      <c r="C28" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="D28" s="93" t="s">
+      <c r="D28" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="112" t="s">
+      <c r="E28" s="137" t="s">
         <v>482</v>
       </c>
-      <c r="F28" s="93" t="s">
+      <c r="F28" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="G28" s="116" t="s">
+      <c r="G28" s="138" t="s">
         <v>483</v>
       </c>
-      <c r="H28" s="105" t="s">
+      <c r="H28" s="139" t="s">
         <v>484</v>
       </c>
-      <c r="I28" s="93" t="s">
-        <v>338</v>
-      </c>
-      <c r="J28" s="93" t="s">
+      <c r="I28" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="J28" s="39" t="s">
         <v>485</v>
       </c>
-      <c r="K28" s="94" t="s">
+      <c r="K28" s="40" t="s">
         <v>486</v>
       </c>
-      <c r="L28" s="93">
+      <c r="L28" s="39">
         <v>1</v>
       </c>
-      <c r="M28" s="95">
+      <c r="M28" s="42">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N28" s="95">
+      <c r="N28" s="42">
         <v>100</v>
       </c>
-      <c r="O28" s="96" t="s">
+      <c r="O28" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P28" s="95">
+      <c r="P28" s="42">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="Q28" s="95">
+      <c r="Q28" s="42">
         <f t="shared" ref="Q28" si="17">N28*P28</f>
         <v>0.33999999999999997</v>
       </c>
-      <c r="R28" s="106" t="s">
+      <c r="R28" s="129" t="s">
         <v>487</v>
       </c>
     </row>
     <row r="29" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
-      <c r="B29" s="85">
+      <c r="B29" s="53">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="86" t="s">
+      <c r="C29" s="61" t="s">
         <v>341</v>
       </c>
-      <c r="D29" s="87" t="s">
+      <c r="D29" s="37" t="s">
         <v>488</v>
       </c>
-      <c r="E29" s="88" t="s">
+      <c r="E29" s="38" t="s">
         <v>95</v>
       </c>
-      <c r="F29" s="87" t="s">
+      <c r="F29" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="G29" s="88" t="s">
+      <c r="G29" s="38" t="s">
         <v>212</v>
       </c>
-      <c r="H29" s="87" t="s">
+      <c r="H29" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="I29" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J29" s="87" t="s">
+      <c r="I29" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J29" s="37" t="s">
         <v>389</v>
       </c>
-      <c r="K29" s="88" t="s">
+      <c r="K29" s="38" t="s">
         <v>297</v>
       </c>
-      <c r="L29" s="109">
+      <c r="L29" s="123">
         <v>1</v>
       </c>
-      <c r="M29" s="89">
+      <c r="M29" s="41">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N29" s="119">
+      <c r="N29" s="135">
         <v>30</v>
       </c>
-      <c r="O29" s="90" t="s">
+      <c r="O29" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P29" s="89">
+      <c r="P29" s="41">
         <v>0.2525</v>
       </c>
-      <c r="Q29" s="89">
+      <c r="Q29" s="41">
         <f t="shared" ref="Q29" si="18">P29*N29</f>
         <v>7.5750000000000002</v>
       </c>
-      <c r="R29" s="91" t="s">
+      <c r="R29" s="136" t="s">
         <v>489</v>
       </c>
     </row>
     <row r="30" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
-      <c r="B30" s="113">
+      <c r="B30" s="53">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="114" t="s">
+      <c r="C30" s="140" t="s">
         <v>341</v>
       </c>
-      <c r="D30" s="115" t="s">
+      <c r="D30" s="141" t="s">
         <v>20</v>
       </c>
-      <c r="E30" s="116" t="s">
+      <c r="E30" s="138" t="s">
         <v>96</v>
       </c>
-      <c r="F30" s="115" t="s">
+      <c r="F30" s="141" t="s">
         <v>158</v>
       </c>
-      <c r="G30" s="116" t="s">
+      <c r="G30" s="138" t="s">
         <v>213</v>
       </c>
-      <c r="H30" s="115" t="s">
+      <c r="H30" s="141" t="s">
         <v>250</v>
       </c>
-      <c r="I30" s="115" t="s">
-        <v>338</v>
-      </c>
-      <c r="J30" s="115" t="s">
+      <c r="I30" s="141" t="s">
+        <v>338</v>
+      </c>
+      <c r="J30" s="141" t="s">
         <v>390</v>
       </c>
-      <c r="K30" s="116" t="s">
+      <c r="K30" s="138" t="s">
         <v>298</v>
       </c>
-      <c r="L30" s="115">
+      <c r="L30" s="141">
         <v>1</v>
       </c>
-      <c r="M30" s="117">
+      <c r="M30" s="142">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N30" s="117">
+      <c r="N30" s="142">
         <v>0</v>
       </c>
-      <c r="O30" s="118" t="s">
+      <c r="O30" s="143" t="s">
         <v>368</v>
       </c>
-      <c r="P30" s="117">
+      <c r="P30" s="142">
         <v>4.1999999999999997E-3</v>
       </c>
-      <c r="Q30" s="117">
+      <c r="Q30" s="142">
         <f t="shared" ref="Q30" si="19">N30*P30</f>
         <v>0</v>
       </c>
-      <c r="R30" s="106" t="s">
+      <c r="R30" s="129" t="s">
         <v>481</v>
       </c>
     </row>
@@ -4798,58 +4816,58 @@
     </row>
     <row r="34" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
-      <c r="B34" s="120">
+      <c r="B34" s="53">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="121" t="s">
+      <c r="C34" s="109" t="s">
         <v>341</v>
       </c>
-      <c r="D34" s="122" t="s">
+      <c r="D34" s="110" t="s">
         <v>24</v>
       </c>
-      <c r="E34" s="123" t="s">
+      <c r="E34" s="111" t="s">
         <v>100</v>
       </c>
-      <c r="F34" s="122" t="s">
+      <c r="F34" s="110" t="s">
         <v>160</v>
       </c>
-      <c r="G34" s="123" t="s">
+      <c r="G34" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="H34" s="122" t="s">
+      <c r="H34" s="110" t="s">
         <v>254</v>
       </c>
-      <c r="I34" s="122" t="s">
+      <c r="I34" s="110" t="s">
         <v>395</v>
       </c>
-      <c r="J34" s="122" t="s">
+      <c r="J34" s="110" t="s">
         <v>394</v>
       </c>
-      <c r="K34" s="123" t="s">
+      <c r="K34" s="111" t="s">
         <v>287</v>
       </c>
-      <c r="L34" s="122">
+      <c r="L34" s="110">
         <v>1</v>
       </c>
-      <c r="M34" s="124">
+      <c r="M34" s="112">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N34" s="124">
+      <c r="N34" s="112">
         <v>0</v>
       </c>
-      <c r="O34" s="125" t="s">
+      <c r="O34" s="113" t="s">
         <v>368</v>
       </c>
-      <c r="P34" s="124">
+      <c r="P34" s="112">
         <v>9.1899999999999996E-2</v>
       </c>
-      <c r="Q34" s="124">
+      <c r="Q34" s="112">
         <f t="shared" ref="Q34" si="23">N34*P34</f>
         <v>0</v>
       </c>
-      <c r="R34" s="124" t="s">
+      <c r="R34" s="112" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5020,115 +5038,115 @@
     </row>
     <row r="38" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
-      <c r="B38" s="85">
+      <c r="B38" s="53">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="92" t="s">
+      <c r="C38" s="60" t="s">
         <v>342</v>
       </c>
-      <c r="D38" s="93" t="s">
-        <v>509</v>
-      </c>
-      <c r="E38" s="94" t="s">
+      <c r="D38" s="39" t="s">
+        <v>507</v>
+      </c>
+      <c r="E38" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="F38" s="93" t="s">
+      <c r="F38" s="39" t="s">
         <v>167</v>
       </c>
-      <c r="G38" s="94" t="s">
+      <c r="G38" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="H38" s="93" t="s">
+      <c r="H38" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="I38" s="93" t="s">
+      <c r="I38" s="39" t="s">
         <v>304</v>
       </c>
-      <c r="J38" s="93" t="s">
+      <c r="J38" s="39" t="s">
         <v>399</v>
       </c>
-      <c r="K38" s="94" t="s">
-        <v>338</v>
-      </c>
-      <c r="L38" s="108">
+      <c r="K38" s="40" t="s">
+        <v>338</v>
+      </c>
+      <c r="L38" s="127">
         <v>2</v>
       </c>
-      <c r="M38" s="95">
+      <c r="M38" s="42">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N38" s="107">
+      <c r="N38" s="128">
         <v>60</v>
       </c>
-      <c r="O38" s="96" t="s">
+      <c r="O38" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P38" s="95">
+      <c r="P38" s="42">
         <v>2.8899999999999999E-2</v>
       </c>
-      <c r="Q38" s="95">
+      <c r="Q38" s="42">
         <f t="shared" ref="Q38" si="27">N38*P38</f>
         <v>1.734</v>
       </c>
-      <c r="R38" s="91" t="s">
-        <v>510</v>
+      <c r="R38" s="144" t="s">
+        <v>508</v>
       </c>
     </row>
     <row r="39" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
-      <c r="B39" s="67">
+      <c r="B39" s="53">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="61" t="s">
         <v>342</v>
       </c>
-      <c r="D39" s="69" t="s">
+      <c r="D39" s="37" t="s">
         <v>472</v>
       </c>
-      <c r="E39" s="70" t="s">
+      <c r="E39" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="F39" s="69" t="s">
+      <c r="F39" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="G39" s="70" t="s">
+      <c r="G39" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="H39" s="69" t="s">
+      <c r="H39" s="37" t="s">
         <v>260</v>
       </c>
-      <c r="I39" s="69" t="s">
+      <c r="I39" s="37" t="s">
         <v>401</v>
       </c>
-      <c r="J39" s="69" t="s">
+      <c r="J39" s="37" t="s">
         <v>402</v>
       </c>
-      <c r="K39" s="70" t="s">
-        <v>338</v>
-      </c>
-      <c r="L39" s="110">
+      <c r="K39" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="L39" s="123">
         <v>9</v>
       </c>
-      <c r="M39" s="71">
+      <c r="M39" s="41">
         <f t="shared" si="1"/>
         <v>180</v>
       </c>
-      <c r="N39" s="139">
+      <c r="N39" s="135">
         <v>190</v>
       </c>
-      <c r="O39" s="72" t="s">
+      <c r="O39" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P39" s="71">
+      <c r="P39" s="41">
         <v>0.12590000000000001</v>
       </c>
-      <c r="Q39" s="71">
+      <c r="Q39" s="41">
         <f t="shared" ref="Q39" si="28">P39*N39</f>
         <v>23.921000000000003</v>
       </c>
-      <c r="R39" s="73" t="s">
+      <c r="R39" s="136" t="s">
         <v>473</v>
       </c>
     </row>
@@ -5244,7 +5262,7 @@
     </row>
     <row r="42" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
-      <c r="B42" s="67">
+      <c r="B42" s="53">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
@@ -5301,58 +5319,58 @@
     </row>
     <row r="43" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
-      <c r="B43" s="67">
+      <c r="B43" s="53">
         <f>ROW(B43) - ROW($B$9)</f>
         <v>34</v>
       </c>
-      <c r="C43" s="68" t="s">
+      <c r="C43" s="61" t="s">
         <v>345</v>
       </c>
-      <c r="D43" s="69" t="s">
+      <c r="D43" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E43" s="70" t="s">
+      <c r="E43" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="F43" s="69" t="s">
+      <c r="F43" s="37" t="s">
         <v>332</v>
       </c>
-      <c r="G43" s="70" t="s">
+      <c r="G43" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="H43" s="69" t="s">
+      <c r="H43" s="37" t="s">
         <v>263</v>
       </c>
-      <c r="I43" s="69" t="s">
+      <c r="I43" s="37" t="s">
         <v>408</v>
       </c>
-      <c r="J43" s="69" t="s">
+      <c r="J43" s="37" t="s">
         <v>409</v>
       </c>
-      <c r="K43" s="70" t="s">
-        <v>338</v>
-      </c>
-      <c r="L43" s="69">
+      <c r="K43" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="L43" s="37">
         <v>2</v>
       </c>
-      <c r="M43" s="71">
+      <c r="M43" s="41">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N43" s="71">
+      <c r="N43" s="41">
         <v>42</v>
       </c>
-      <c r="O43" s="72" t="s">
+      <c r="O43" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P43" s="71">
+      <c r="P43" s="41">
         <v>0.65639999999999998</v>
       </c>
-      <c r="Q43" s="71">
+      <c r="Q43" s="41">
         <f t="shared" ref="Q43" si="32">P43*N43</f>
         <v>27.5688</v>
       </c>
-      <c r="R43" s="73" t="s">
+      <c r="R43" s="136" t="s">
         <v>400</v>
       </c>
     </row>
@@ -5523,59 +5541,59 @@
     </row>
     <row r="47" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
-      <c r="B47" s="85">
+      <c r="B47" s="53">
         <f>ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
-      <c r="C47" s="86" t="s">
+      <c r="C47" s="61" t="s">
         <v>343</v>
       </c>
-      <c r="D47" s="87" t="s">
+      <c r="D47" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="E47" s="88" t="s">
+      <c r="E47" s="38" t="s">
+        <v>501</v>
+      </c>
+      <c r="F47" s="37" t="s">
+        <v>332</v>
+      </c>
+      <c r="G47" s="38" t="s">
+        <v>502</v>
+      </c>
+      <c r="H47" s="126" t="s">
         <v>503</v>
       </c>
-      <c r="F47" s="87" t="s">
-        <v>332</v>
-      </c>
-      <c r="G47" s="88" t="s">
+      <c r="I47" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J47" s="37" t="s">
         <v>504</v>
       </c>
-      <c r="H47" s="97" t="s">
+      <c r="K47" s="38" t="s">
         <v>505</v>
       </c>
-      <c r="I47" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J47" s="87" t="s">
-        <v>506</v>
-      </c>
-      <c r="K47" s="88" t="s">
-        <v>507</v>
-      </c>
-      <c r="L47" s="87">
+      <c r="L47" s="37">
         <v>1</v>
       </c>
-      <c r="M47" s="89">
+      <c r="M47" s="41">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N47" s="119">
+      <c r="N47" s="135">
         <v>25</v>
       </c>
-      <c r="O47" s="90" t="s">
+      <c r="O47" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P47" s="89">
+      <c r="P47" s="41">
         <v>0.1012</v>
       </c>
-      <c r="Q47" s="89">
+      <c r="Q47" s="41">
         <f t="shared" ref="Q47" si="36">P47*N47</f>
         <v>2.5299999999999998</v>
       </c>
-      <c r="R47" s="106" t="s">
-        <v>508</v>
+      <c r="R47" s="124" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -5885,7 +5903,7 @@
       <c r="K53" s="70" t="s">
         <v>338</v>
       </c>
-      <c r="L53" s="110">
+      <c r="L53" s="106">
         <v>4</v>
       </c>
       <c r="M53" s="71">
@@ -6248,7 +6266,7 @@
       <c r="C60" s="92" t="s">
         <v>349</v>
       </c>
-      <c r="D60" s="105" t="s">
+      <c r="D60" s="101" t="s">
         <v>461</v>
       </c>
       <c r="E60" s="94" t="s">
@@ -6270,14 +6288,14 @@
       <c r="K60" s="94" t="s">
         <v>313</v>
       </c>
-      <c r="L60" s="108">
+      <c r="L60" s="104">
         <v>1</v>
       </c>
       <c r="M60" s="95">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N60" s="107">
+      <c r="N60" s="103">
         <v>100</v>
       </c>
       <c r="O60" s="96" t="s">
@@ -6290,7 +6308,7 @@
         <f t="shared" ref="Q60:Q61" si="50">N60*P60</f>
         <v>0.15</v>
       </c>
-      <c r="R60" s="106" t="s">
+      <c r="R60" s="102" t="s">
         <v>462</v>
       </c>
     </row>
@@ -6327,17 +6345,17 @@
       <c r="K61" s="87" t="s">
         <v>466</v>
       </c>
-      <c r="L61" s="109">
+      <c r="L61" s="105">
         <v>8</v>
       </c>
       <c r="M61" s="87">
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="N61" s="107">
+      <c r="N61" s="103">
         <v>100</v>
       </c>
-      <c r="O61" s="111" t="s">
+      <c r="O61" s="107" t="s">
         <v>368</v>
       </c>
       <c r="P61" s="87">
@@ -6347,7 +6365,7 @@
         <f t="shared" si="50"/>
         <v>0.11</v>
       </c>
-      <c r="R61" s="106" t="s">
+      <c r="R61" s="102" t="s">
         <v>467</v>
       </c>
     </row>
@@ -6800,7 +6818,7 @@
       <c r="C70" s="61" t="s">
         <v>349</v>
       </c>
-      <c r="D70" s="69" t="s">
+      <c r="D70" s="37" t="s">
         <v>435</v>
       </c>
       <c r="E70" s="38" t="s">
@@ -6824,7 +6842,7 @@
       <c r="K70" s="38" t="s">
         <v>322</v>
       </c>
-      <c r="L70" s="110">
+      <c r="L70" s="123">
         <v>2</v>
       </c>
       <c r="M70" s="41">
@@ -7019,111 +7037,111 @@
         <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
-      <c r="C74" s="86" t="s">
+      <c r="C74" s="61" t="s">
         <v>349</v>
       </c>
-      <c r="D74" s="87" t="s">
+      <c r="D74" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="E74" s="132" t="s">
+      <c r="E74" s="125" t="s">
+        <v>495</v>
+      </c>
+      <c r="F74" s="145" t="s">
+        <v>496</v>
+      </c>
+      <c r="G74" s="38" t="s">
         <v>497</v>
       </c>
-      <c r="F74" s="138" t="s">
+      <c r="H74" s="126" t="s">
+        <v>273</v>
+      </c>
+      <c r="I74" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="J74" s="37" t="s">
         <v>498</v>
       </c>
-      <c r="G74" s="88" t="s">
+      <c r="K74" s="38" t="s">
         <v>499</v>
       </c>
-      <c r="H74" s="97" t="s">
-        <v>273</v>
-      </c>
-      <c r="I74" s="87" t="s">
-        <v>338</v>
-      </c>
-      <c r="J74" s="87" t="s">
-        <v>500</v>
-      </c>
-      <c r="K74" s="88" t="s">
-        <v>501</v>
-      </c>
-      <c r="L74" s="87">
+      <c r="L74" s="37">
         <v>1</v>
       </c>
-      <c r="M74" s="89">
+      <c r="M74" s="41">
         <f t="shared" ref="M74:M92" si="63">L74*20</f>
         <v>20</v>
       </c>
-      <c r="N74" s="119">
+      <c r="N74" s="135">
         <v>50</v>
       </c>
-      <c r="O74" s="90" t="s">
+      <c r="O74" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P74" s="89">
+      <c r="P74" s="41">
         <v>3.8E-3</v>
       </c>
-      <c r="Q74" s="89">
+      <c r="Q74" s="41">
         <f t="shared" ref="Q74" si="64">P74*N74</f>
         <v>0.19</v>
       </c>
-      <c r="R74" s="106" t="s">
-        <v>502</v>
+      <c r="R74" s="124" t="s">
+        <v>500</v>
       </c>
     </row>
     <row r="75" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1"/>
-      <c r="B75" s="113">
+      <c r="B75" s="108">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C75" s="114" t="s">
+      <c r="C75" s="140" t="s">
         <v>349</v>
       </c>
-      <c r="D75" s="115" t="s">
+      <c r="D75" s="141" t="s">
         <v>60</v>
       </c>
-      <c r="E75" s="116" t="s">
+      <c r="E75" s="138" t="s">
         <v>138</v>
       </c>
-      <c r="F75" s="115" t="s">
+      <c r="F75" s="141" t="s">
         <v>182</v>
       </c>
-      <c r="G75" s="116" t="s">
+      <c r="G75" s="138" t="s">
         <v>239</v>
       </c>
-      <c r="H75" s="115" t="s">
+      <c r="H75" s="141" t="s">
         <v>272</v>
       </c>
-      <c r="I75" s="115" t="s">
-        <v>338</v>
-      </c>
-      <c r="J75" s="115" t="s">
-        <v>338</v>
-      </c>
-      <c r="K75" s="116" t="s">
+      <c r="I75" s="141" t="s">
+        <v>338</v>
+      </c>
+      <c r="J75" s="141" t="s">
+        <v>338</v>
+      </c>
+      <c r="K75" s="138" t="s">
         <v>326</v>
       </c>
-      <c r="L75" s="115">
+      <c r="L75" s="141">
         <v>1</v>
       </c>
-      <c r="M75" s="117">
+      <c r="M75" s="142">
         <f t="shared" si="63"/>
         <v>20</v>
       </c>
-      <c r="N75" s="117">
+      <c r="N75" s="142">
         <v>0</v>
       </c>
-      <c r="O75" s="118" t="s">
+      <c r="O75" s="143" t="s">
         <v>413</v>
       </c>
-      <c r="P75" s="117">
+      <c r="P75" s="142">
         <v>1.8589999999999999E-2</v>
       </c>
-      <c r="Q75" s="117">
+      <c r="Q75" s="142">
         <f t="shared" ref="Q75" si="65">N75*P75</f>
         <v>0</v>
       </c>
-      <c r="R75" s="106" t="s">
+      <c r="R75" s="129" t="s">
         <v>481</v>
       </c>
     </row>
@@ -7298,55 +7316,55 @@
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C79" s="92" t="s">
+      <c r="C79" s="60" t="s">
         <v>349</v>
       </c>
-      <c r="D79" s="93" t="s">
-        <v>495</v>
-      </c>
-      <c r="E79" s="94" t="s">
+      <c r="D79" s="39" t="s">
+        <v>493</v>
+      </c>
+      <c r="E79" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="F79" s="93" t="s">
+      <c r="F79" s="39" t="s">
         <v>182</v>
       </c>
-      <c r="G79" s="94" t="s">
+      <c r="G79" s="40" t="s">
         <v>241</v>
       </c>
-      <c r="H79" s="93" t="s">
+      <c r="H79" s="39" t="s">
         <v>250</v>
       </c>
-      <c r="I79" s="93" t="s">
-        <v>338</v>
-      </c>
-      <c r="J79" s="93" t="s">
+      <c r="I79" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="J79" s="39" t="s">
         <v>443</v>
       </c>
-      <c r="K79" s="94" t="s">
+      <c r="K79" s="40" t="s">
         <v>330</v>
       </c>
-      <c r="L79" s="93">
+      <c r="L79" s="39">
         <v>6</v>
       </c>
-      <c r="M79" s="95">
+      <c r="M79" s="42">
         <f t="shared" si="63"/>
         <v>120</v>
       </c>
-      <c r="N79" s="95">
+      <c r="N79" s="42">
         <v>200</v>
       </c>
-      <c r="O79" s="96" t="s">
+      <c r="O79" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P79" s="95">
+      <c r="P79" s="42">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="Q79" s="95">
+      <c r="Q79" s="42">
         <f t="shared" ref="Q79" si="69">N79*P79</f>
         <v>0.24</v>
       </c>
-      <c r="R79" s="106" t="s">
-        <v>496</v>
+      <c r="R79" s="129" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="80" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -7569,54 +7587,54 @@
         <f>ROW(B84) - ROW($B$9)</f>
         <v>75</v>
       </c>
-      <c r="C84" s="86" t="s">
+      <c r="C84" s="61" t="s">
         <v>353</v>
       </c>
-      <c r="D84" s="87" t="s">
+      <c r="D84" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="E84" s="88" t="s">
+      <c r="E84" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="F84" s="87" t="s">
+      <c r="F84" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="G84" s="88" t="s">
+      <c r="G84" s="38" t="s">
         <v>242</v>
       </c>
-      <c r="H84" s="87" t="s">
+      <c r="H84" s="37" t="s">
         <v>278</v>
       </c>
-      <c r="I84" s="87" t="s">
+      <c r="I84" s="37" t="s">
         <v>445</v>
       </c>
-      <c r="J84" s="87" t="s">
+      <c r="J84" s="37" t="s">
         <v>446</v>
       </c>
-      <c r="K84" s="88" t="s">
-        <v>338</v>
-      </c>
-      <c r="L84" s="87">
+      <c r="K84" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="L84" s="37">
         <v>1</v>
       </c>
-      <c r="M84" s="89">
+      <c r="M84" s="41">
         <f t="shared" si="63"/>
         <v>20</v>
       </c>
-      <c r="N84" s="89">
+      <c r="N84" s="41">
         <v>21</v>
       </c>
-      <c r="O84" s="90" t="s">
+      <c r="O84" s="64" t="s">
         <v>368</v>
       </c>
-      <c r="P84" s="89">
+      <c r="P84" s="41">
         <v>1.3939999999999999</v>
       </c>
-      <c r="Q84" s="89">
+      <c r="Q84" s="41">
         <f t="shared" ref="Q84" si="75">P84*N84</f>
         <v>29.273999999999997</v>
       </c>
-      <c r="R84" s="91" t="s">
+      <c r="R84" s="136" t="s">
         <v>474</v>
       </c>
     </row>
@@ -7626,54 +7644,54 @@
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="C85" s="92" t="s">
+      <c r="C85" s="60" t="s">
         <v>353</v>
       </c>
-      <c r="D85" s="93" t="s">
+      <c r="D85" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="E85" s="94" t="s">
+      <c r="E85" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="F85" s="93" t="s">
+      <c r="F85" s="39" t="s">
         <v>189</v>
       </c>
-      <c r="G85" s="94" t="s">
+      <c r="G85" s="40" t="s">
         <v>243</v>
       </c>
-      <c r="H85" s="93" t="s">
+      <c r="H85" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="I85" s="93" t="s">
+      <c r="I85" s="39" t="s">
         <v>448</v>
       </c>
-      <c r="J85" s="93" t="s">
+      <c r="J85" s="39" t="s">
         <v>449</v>
       </c>
-      <c r="K85" s="94" t="s">
-        <v>338</v>
-      </c>
-      <c r="L85" s="93">
+      <c r="K85" s="40" t="s">
+        <v>338</v>
+      </c>
+      <c r="L85" s="39">
         <v>1</v>
       </c>
-      <c r="M85" s="95">
+      <c r="M85" s="42">
         <f t="shared" si="63"/>
         <v>20</v>
       </c>
-      <c r="N85" s="95">
+      <c r="N85" s="42">
         <v>21</v>
       </c>
-      <c r="O85" s="96" t="s">
+      <c r="O85" s="65" t="s">
         <v>368</v>
       </c>
-      <c r="P85" s="95">
+      <c r="P85" s="42">
         <v>0.69430000000000003</v>
       </c>
-      <c r="Q85" s="95">
+      <c r="Q85" s="42">
         <f t="shared" ref="Q85" si="76">N85*P85</f>
         <v>14.580300000000001</v>
       </c>
-      <c r="R85" s="91" t="s">
+      <c r="R85" s="144" t="s">
         <v>447</v>
       </c>
     </row>
@@ -7789,59 +7807,59 @@
     </row>
     <row r="88" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1"/>
-      <c r="B88" s="126">
+      <c r="B88" s="114">
         <f>ROW(B88) - ROW($B$9)</f>
         <v>79</v>
       </c>
-      <c r="C88" s="127" t="s">
+      <c r="C88" s="115" t="s">
         <v>353</v>
       </c>
-      <c r="D88" s="128" t="s">
+      <c r="D88" s="116" t="s">
         <v>72</v>
       </c>
-      <c r="E88" s="129" t="s">
+      <c r="E88" s="117" t="s">
         <v>151</v>
       </c>
-      <c r="F88" s="128" t="s">
+      <c r="F88" s="116" t="s">
         <v>192</v>
       </c>
-      <c r="G88" s="129" t="s">
+      <c r="G88" s="117" t="s">
         <v>245</v>
       </c>
-      <c r="H88" s="128" t="s">
+      <c r="H88" s="116" t="s">
         <v>279</v>
       </c>
-      <c r="I88" s="128" t="s">
-        <v>338</v>
-      </c>
-      <c r="J88" s="128" t="s">
+      <c r="I88" s="116" t="s">
+        <v>338</v>
+      </c>
+      <c r="J88" s="116" t="s">
         <v>451</v>
       </c>
-      <c r="K88" s="129" t="s">
-        <v>338</v>
-      </c>
-      <c r="L88" s="128">
+      <c r="K88" s="117" t="s">
+        <v>338</v>
+      </c>
+      <c r="L88" s="116">
         <v>1</v>
       </c>
-      <c r="M88" s="130">
+      <c r="M88" s="118">
         <f t="shared" si="63"/>
         <v>20</v>
       </c>
-      <c r="N88" s="130">
+      <c r="N88" s="118">
         <v>21</v>
       </c>
-      <c r="O88" s="131" t="s">
+      <c r="O88" s="119" t="s">
         <v>368</v>
       </c>
-      <c r="P88" s="130">
+      <c r="P88" s="118">
         <v>7.4638</v>
       </c>
-      <c r="Q88" s="130">
+      <c r="Q88" s="118">
         <f t="shared" ref="Q88" si="79">P88*N88</f>
         <v>156.7398</v>
       </c>
-      <c r="R88" s="130" t="s">
-        <v>512</v>
+      <c r="R88" s="118" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="89" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7932,7 +7950,7 @@
       <c r="K90" s="88" t="s">
         <v>338</v>
       </c>
-      <c r="L90" s="109">
+      <c r="L90" s="105">
         <v>2</v>
       </c>
       <c r="M90" s="89">
@@ -8010,7 +8028,7 @@
         <v>74.171999999999997</v>
       </c>
       <c r="R91" s="91" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="92" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8085,13 +8103,13 @@
       <c r="L93" s="36"/>
       <c r="M93" s="36"/>
       <c r="N93" s="36"/>
-      <c r="O93" s="100" t="s">
+      <c r="O93" s="99" t="s">
         <v>458</v>
       </c>
-      <c r="P93" s="98"/>
-      <c r="Q93" s="98">
+      <c r="P93" s="97"/>
+      <c r="Q93" s="97">
         <f>SUM(Q10:Q92)</f>
-        <v>963.24749999999995</v>
+        <v>963.91150000000016</v>
       </c>
       <c r="R93" s="44"/>
     </row>
@@ -8112,13 +8130,13 @@
       <c r="L94" s="9"/>
       <c r="M94" s="9"/>
       <c r="N94" s="9"/>
-      <c r="O94" s="101" t="s">
+      <c r="O94" s="100" t="s">
         <v>459</v>
       </c>
-      <c r="P94" s="99"/>
-      <c r="Q94" s="99">
+      <c r="P94" s="98"/>
+      <c r="Q94" s="98">
         <f>Q93/20</f>
-        <v>48.162374999999997</v>
+        <v>48.195575000000005</v>
       </c>
       <c r="R94" s="45"/>
     </row>

</xml_diff>